<commit_message>
lk chuc nang dang nhap va dang ky voi database
</commit_message>
<xml_diff>
--- a/DOCX/TextCases.xlsx
+++ b/DOCX/TextCases.xlsx
@@ -5,15 +5,26 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI Gaming\NP-CHAT-01\DOCX\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202134A5-D848-41FA-928F-D782D09DB0F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C9D9F8-EDD9-467A-9C79-164842CDDAE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="TC001" sheetId="2" r:id="rId2"/>
+    <sheet name="TC002" sheetId="3" r:id="rId3"/>
+    <sheet name="TC003" sheetId="4" r:id="rId4"/>
+    <sheet name="TC004" sheetId="5" r:id="rId5"/>
+    <sheet name="TC007" sheetId="6" r:id="rId6"/>
+    <sheet name="TC008" sheetId="7" r:id="rId7"/>
+    <sheet name="TC009" sheetId="8" r:id="rId8"/>
+    <sheet name="TC010" sheetId="9" r:id="rId9"/>
+    <sheet name="TC012" sheetId="12" r:id="rId10"/>
+    <sheet name="TC014" sheetId="10" r:id="rId11"/>
+    <sheet name="TC015" sheetId="11" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Cases'!$A$1:$J$12</definedName>
@@ -774,6 +785,738 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>133350</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>458266</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>634</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65F78C3B-2084-F7E0-0594-7D6276CF92CD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="133350" y="28575"/>
+          <a:ext cx="7640116" cy="4544059"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>485775</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>162986</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>19684</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17EF0AC9-ED8D-7FA1-1315-EDE40F7D015D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7800975" y="47625"/>
+          <a:ext cx="7602011" cy="4544059"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>91737</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A7955D3-6335-281C-28EC-1DD081089659}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="28575" y="9525"/>
+          <a:ext cx="9115425" cy="4463712"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>117465</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B31F663B-F9D8-8689-392D-F82A7C76D2ED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="4629150"/>
+          <a:ext cx="12919065" cy="4791075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>57862</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C50448A5-0D17-6A6B-792E-B0D978460516}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="28575" y="19050"/>
+          <a:ext cx="12221287" cy="4143375"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>40664</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{815DEBE5-3E05-5F48-3389-85032957A1BA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="15890264" cy="4600575"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>97471</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>76841</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38E6BE8D-671D-61E8-D030-AED6BFEAFFF1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="28575" y="4629150"/>
+          <a:ext cx="15918496" cy="4591691"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>247650</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>582093</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>48262</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11EE47EB-BD62-62C3-6B28-9C93378234B0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="247650" y="57150"/>
+          <a:ext cx="7649643" cy="4563112"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>95250</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>249883</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>38840</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B6F772A-248D-210D-679C-1847BD2DA7F0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="95250" y="66675"/>
+          <a:ext cx="16004233" cy="5306165"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>168251</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A53F454E-99EA-F035-390A-6369D66EF44B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="13134975" cy="6645251"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>68</xdr:row>
+      <xdr:rowOff>86239</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4920592F-CC7B-9F69-7EF9-08A96E2E1B88}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="7277100"/>
+          <a:ext cx="13144500" cy="5763139"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>602286</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>162665</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B36973B1-59D8-1C39-6363-9E9F0CE0E3F4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="15842286" cy="5306165"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>173346</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>153033</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B90F25B-6004-EA50-6608-14B3DF2A6E7E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="13584546" cy="4534533"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>335123</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>181665</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{98198E84-06C8-04C6-F5FC-E2310414F3E4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="12527123" cy="4944165"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>22411</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>151655</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB822D6F-9ABD-92E5-2C6B-EBDE31D577E4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="10914529" cy="5485655"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1645,4 +2388,114 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A1F8565-5620-4AB0-B357-72D6C1038C07}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF758F81-9343-40C5-8D0A-4D4E65741192}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F84AA9AC-75DC-42DC-9B12-2E32C4001131}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FEE79D7-B28A-4F93-82BF-CEFD86BE5907}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{578FACE4-58F9-4840-9A3E-381EF6BB51B6}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBB1AB42-D32B-4A79-B5B4-8DC6CDBD7F2E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{768FFEFB-8C25-4FEE-BBA5-E0E38EC6029E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C92D74A-F663-47CD-9BB6-FD01B89C79D7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DBF5620-BCAC-4081-83DD-B60E09736327}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD2D833E-8A31-40C2-A007-1BB3390B623D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C7597E0-1AB1-494D-A59C-EA5CAA1BA460}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>